<commit_message>
feat(reports): source Distribution Rewards from settle-dr-dune (#139)
Co-authored-by: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-03/grove_settlement_march_2026.xlsx
+++ b/settlements/grove/2026-03/grove_settlement_march_2026.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -506,168 +506,178 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" s="4" t="n">
-        <v>1062588.479948548</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>+ distribution_rewards (settle-dr-dune)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>191719.25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" s="4" t="n">
+        <v>1254307.729948548</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Sky side</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CoF on utilized (BR × Net_Subs)</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>3056810.760658033</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>CoF on utilized (BR × Net_Subs)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>3056810.760658033</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>+ SDE revenue (Sky-Direct, full to Sky)</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B11" s="3" t="n">
         <v>3251383.753143241</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" s="4" t="n">
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" s="4" t="n">
         <v>6308194.513801275</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Sky Revenue (max) — BR × full ilk debt, no deductions</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CoF on Net_Subs (actual BR × utilized)</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>3056810.760658033</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>CoF on Net_Subs (actual BR × utilized)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>3056810.760658033</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>reduction from idle/SDE deductions</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B16" s="3" t="n">
         <v>-4916099.3356033</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" s="4" t="n">
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" s="4" t="n">
         <v>7972910.096261334</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Comparison (Grove-style "Profit to Grove")</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>prime_agent_revenue</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>1056301.360503078</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>prime_agent_revenue</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1056301.360503078</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>− CoF (deducted per-venue in display)</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B21" s="3" t="n">
         <v>-3056810.760658033</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" s="4" t="n">
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" s="4" t="n">
         <v>-2000509.400154955</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-03-01 → 2026-03-31 (31 days)</t>
-        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Pin blocks</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>avalanche_c=81789468, base=44106126, ethereum=24781026, monad=4, plume=58679343</t>
+          <t>2026-03-01 → 2026-03-31 (31 days)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Generated</t>
+          <t>Pin blocks</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-23T21:34:39+00:00</t>
+          <t>avalanche_c=81789468, base=44106126, ethereum=24781026, monad=4, plume=58679343</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-06-23T22:21:59+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>

</xml_diff>